<commit_message>
Daily recap, matchup updates, learning and research 2026-08-21
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-21.xlsx
+++ b/data/k-props/2026-08-21.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="100">
   <si>
     <t>date</t>
   </si>
@@ -145,6 +145,9 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -181,6 +184,9 @@
     <t>Cam Schlittler</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>Logan Webb</t>
   </si>
   <si>
@@ -190,10 +196,16 @@
     <t>Sonny Gray</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t>Brad Lord</t>
   </si>
   <si>
     <t>Washington Nationals @ Miami Marlins</t>
+  </si>
+  <si>
+    <t>W</t>
   </si>
   <si>
     <t>Ryan Gusto</t>
@@ -880,17 +892,23 @@
       <c r="Y2">
         <v>0.9358</v>
       </c>
+      <c r="Z2">
+        <v>6</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>-0.01</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>7.49</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.3299</v>
@@ -900,6 +918,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>-1.49</v>
+      </c>
+      <c r="AJ2">
+        <v>1.49</v>
+      </c>
+      <c r="AK2">
+        <v>-1.49</v>
+      </c>
+      <c r="AL2">
+        <v>1.49</v>
       </c>
       <c r="AM2">
         <v>7.49</v>
@@ -910,7 +940,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>9.5</v>
@@ -981,17 +1011,23 @@
       <c r="Y3">
         <v>1.0407</v>
       </c>
+      <c r="Z3">
+        <v>6</v>
+      </c>
       <c r="AA3" t="s">
         <v>44</v>
       </c>
+      <c r="AB3">
+        <v>0.3</v>
+      </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD3">
         <v>9.8</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.3908</v>
@@ -1001,6 +1037,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-3.8</v>
+      </c>
+      <c r="AJ3">
+        <v>3.8</v>
+      </c>
+      <c r="AK3">
+        <v>-3.8</v>
+      </c>
+      <c r="AL3">
+        <v>3.8</v>
       </c>
       <c r="AM3">
         <v>9.8</v>
@@ -1011,7 +1059,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C4">
         <v>3.5</v>
@@ -1023,7 +1071,7 @@
         <v>123</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G4">
         <v>823420</v>
@@ -1082,17 +1130,23 @@
       <c r="Y4">
         <v>0.922</v>
       </c>
+      <c r="Z4">
+        <v>3</v>
+      </c>
       <c r="AA4" t="s">
         <v>44</v>
       </c>
+      <c r="AB4">
+        <v>-0.39</v>
+      </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD4">
         <v>3.11</v>
       </c>
       <c r="AE4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF4">
         <v>0.2253</v>
@@ -1102,6 +1156,18 @@
       </c>
       <c r="AH4">
         <v>0</v>
+      </c>
+      <c r="AI4">
+        <v>-0.11</v>
+      </c>
+      <c r="AJ4">
+        <v>0.11</v>
+      </c>
+      <c r="AK4">
+        <v>-0.11</v>
+      </c>
+      <c r="AL4">
+        <v>0.11</v>
       </c>
       <c r="AM4">
         <v>3.11</v>
@@ -1112,10 +1178,10 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G5">
         <v>823420</v>
@@ -1175,16 +1241,16 @@
         <v>0.9461</v>
       </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD5">
         <v>6.86</v>
       </c>
       <c r="AE5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AF5">
         <v>0.3013</v>
@@ -1204,16 +1270,16 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G6">
         <v>823510</v>
       </c>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I6">
         <v>1.1</v>
@@ -1267,16 +1333,16 @@
         <v>1.0045</v>
       </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD6">
         <v>1.43</v>
       </c>
       <c r="AE6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF6">
         <v>0.2516</v>
@@ -1296,7 +1362,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C7">
         <v>6.5</v>
@@ -1308,7 +1374,7 @@
         <v>-105</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G7">
         <v>823510</v>
@@ -1367,17 +1433,23 @@
       <c r="Y7">
         <v>0.98</v>
       </c>
+      <c r="Z7">
+        <v>4</v>
+      </c>
       <c r="AA7" t="s">
         <v>44</v>
       </c>
+      <c r="AB7">
+        <v>0.7</v>
+      </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD7">
         <v>6.8</v>
       </c>
       <c r="AE7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AF7">
         <v>0.3207</v>
@@ -1387,6 +1459,18 @@
       </c>
       <c r="AH7">
         <v>0.4</v>
+      </c>
+      <c r="AI7">
+        <v>-2.8</v>
+      </c>
+      <c r="AJ7">
+        <v>2.8</v>
+      </c>
+      <c r="AK7">
+        <v>-3.2</v>
+      </c>
+      <c r="AL7">
+        <v>3.2</v>
       </c>
       <c r="AM7">
         <v>7.2</v>
@@ -1397,7 +1481,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C8">
         <v>4.5</v>
@@ -1409,7 +1493,7 @@
         <v>-125</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G8">
         <v>824721</v>
@@ -1468,17 +1552,23 @@
       <c r="Y8">
         <v>0.9943</v>
       </c>
+      <c r="Z8">
+        <v>2</v>
+      </c>
       <c r="AA8" t="s">
         <v>44</v>
       </c>
+      <c r="AB8">
+        <v>-0.3</v>
+      </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD8">
         <v>4.2</v>
       </c>
       <c r="AE8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF8">
         <v>0.1994</v>
@@ -1488,6 +1578,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>-2.2</v>
+      </c>
+      <c r="AJ8">
+        <v>2.2</v>
+      </c>
+      <c r="AK8">
+        <v>-2.2</v>
+      </c>
+      <c r="AL8">
+        <v>2.2</v>
       </c>
       <c r="AM8">
         <v>4.2</v>
@@ -1498,7 +1600,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C9">
         <v>5.5</v>
@@ -1510,7 +1612,7 @@
         <v>-104</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>824721</v>
@@ -1569,17 +1671,23 @@
       <c r="Y9">
         <v>0.9508</v>
       </c>
+      <c r="Z9">
+        <v>6</v>
+      </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="AB9">
+        <v>-0.96</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD9">
         <v>4.54</v>
       </c>
       <c r="AE9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF9">
         <v>0.2228</v>
@@ -1589,6 +1697,18 @@
       </c>
       <c r="AH9">
         <v>0</v>
+      </c>
+      <c r="AI9">
+        <v>1.46</v>
+      </c>
+      <c r="AJ9">
+        <v>1.46</v>
+      </c>
+      <c r="AK9">
+        <v>1.46</v>
+      </c>
+      <c r="AL9">
+        <v>1.46</v>
       </c>
       <c r="AM9">
         <v>4.54</v>
@@ -1599,7 +1719,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C10">
         <v>2.5</v>
@@ -1611,13 +1731,13 @@
         <v>-105</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G10">
         <v>823830</v>
       </c>
       <c r="H10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I10">
         <v>1.7</v>
@@ -1670,17 +1790,23 @@
       <c r="Y10">
         <v>0.8899</v>
       </c>
+      <c r="Z10">
+        <v>1</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>-1.08</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="AD10">
         <v>1.42</v>
       </c>
       <c r="AE10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF10">
         <v>0.2037</v>
@@ -1690,6 +1816,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>-0.42</v>
+      </c>
+      <c r="AJ10">
+        <v>0.42</v>
+      </c>
+      <c r="AK10">
+        <v>-0.42</v>
+      </c>
+      <c r="AL10">
+        <v>0.42</v>
       </c>
       <c r="AM10">
         <v>1.42</v>
@@ -1700,7 +1838,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C11">
         <v>3.5</v>
@@ -1712,13 +1850,13 @@
         <v>135</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G11">
         <v>823830</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I11">
         <v>3.8</v>
@@ -1771,17 +1909,23 @@
       <c r="Y11">
         <v>0.9397</v>
       </c>
+      <c r="Z11">
+        <v>2</v>
+      </c>
       <c r="AA11" t="s">
         <v>44</v>
       </c>
+      <c r="AB11">
+        <v>-0.51</v>
+      </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD11">
         <v>2.99</v>
       </c>
       <c r="AE11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF11">
         <v>0.2029</v>
@@ -1791,6 +1935,18 @@
       </c>
       <c r="AH11">
         <v>0</v>
+      </c>
+      <c r="AI11">
+        <v>-0.99</v>
+      </c>
+      <c r="AJ11">
+        <v>0.99</v>
+      </c>
+      <c r="AK11">
+        <v>-0.99</v>
+      </c>
+      <c r="AL11">
+        <v>0.99</v>
       </c>
       <c r="AM11">
         <v>2.99</v>
@@ -1801,7 +1957,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>5.5</v>
@@ -1813,7 +1969,7 @@
         <v>-146</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G12">
         <v>824800</v>
@@ -1872,17 +2028,23 @@
       <c r="Y12">
         <v>1.0527</v>
       </c>
+      <c r="Z12">
+        <v>6</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="AB12">
+        <v>0.04</v>
       </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD12">
         <v>5.54</v>
       </c>
       <c r="AE12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF12">
         <v>0.199</v>
@@ -1892,6 +2054,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>0.46</v>
+      </c>
+      <c r="AJ12">
+        <v>0.46</v>
+      </c>
+      <c r="AK12">
+        <v>0.46</v>
+      </c>
+      <c r="AL12">
+        <v>0.46</v>
       </c>
       <c r="AM12">
         <v>5.54</v>
@@ -1902,7 +2076,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C13">
         <v>4.5</v>
@@ -1914,7 +2088,7 @@
         <v>-110</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G13">
         <v>824800</v>
@@ -1973,17 +2147,23 @@
       <c r="Y13">
         <v>0.88</v>
       </c>
+      <c r="Z13">
+        <v>6</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="AB13">
+        <v>-1.47</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD13">
         <v>3.03</v>
       </c>
       <c r="AE13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF13">
         <v>0.2186</v>
@@ -1993,6 +2173,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>2.97</v>
+      </c>
+      <c r="AJ13">
+        <v>2.97</v>
+      </c>
+      <c r="AK13">
+        <v>2.97</v>
+      </c>
+      <c r="AL13">
+        <v>2.97</v>
       </c>
       <c r="AM13">
         <v>3.03</v>
@@ -2003,7 +2195,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C14">
         <v>5.5</v>
@@ -2015,7 +2207,7 @@
         <v>120</v>
       </c>
       <c r="F14" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G14">
         <v>824559</v>
@@ -2074,17 +2266,23 @@
       <c r="Y14">
         <v>1.1</v>
       </c>
+      <c r="Z14">
+        <v>4</v>
+      </c>
       <c r="AA14" t="s">
         <v>44</v>
       </c>
+      <c r="AB14">
+        <v>1.86</v>
+      </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD14">
         <v>7.36</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.2408</v>
@@ -2094,6 +2292,18 @@
       </c>
       <c r="AH14">
         <v>0</v>
+      </c>
+      <c r="AI14">
+        <v>-3.36</v>
+      </c>
+      <c r="AJ14">
+        <v>3.36</v>
+      </c>
+      <c r="AK14">
+        <v>-3.36</v>
+      </c>
+      <c r="AL14">
+        <v>3.36</v>
       </c>
       <c r="AM14">
         <v>7.36</v>
@@ -2104,7 +2314,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C15">
         <v>6.5</v>
@@ -2116,7 +2326,7 @@
         <v>-137</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G15">
         <v>824559</v>
@@ -2175,17 +2385,23 @@
       <c r="Y15">
         <v>0.9737</v>
       </c>
+      <c r="Z15">
+        <v>4</v>
+      </c>
       <c r="AA15" t="s">
         <v>44</v>
       </c>
+      <c r="AB15">
+        <v>0.77</v>
+      </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD15">
         <v>6.87</v>
       </c>
       <c r="AE15" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AF15">
         <v>0.281</v>
@@ -2195,6 +2411,18 @@
       </c>
       <c r="AH15">
         <v>0.4</v>
+      </c>
+      <c r="AI15">
+        <v>-2.87</v>
+      </c>
+      <c r="AJ15">
+        <v>2.87</v>
+      </c>
+      <c r="AK15">
+        <v>-3.27</v>
+      </c>
+      <c r="AL15">
+        <v>3.27</v>
       </c>
       <c r="AM15">
         <v>7.27</v>
@@ -2205,7 +2433,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C16">
         <v>4.5</v>
@@ -2217,7 +2445,7 @@
         <v>-120</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G16">
         <v>824072</v>
@@ -2276,17 +2504,23 @@
       <c r="Y16">
         <v>0.9306</v>
       </c>
+      <c r="Z16">
+        <v>3</v>
+      </c>
       <c r="AA16" t="s">
         <v>44</v>
       </c>
+      <c r="AB16">
+        <v>-0.5</v>
+      </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD16">
         <v>4</v>
       </c>
       <c r="AE16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF16">
         <v>0.2125</v>
@@ -2296,6 +2530,18 @@
       </c>
       <c r="AH16">
         <v>0</v>
+      </c>
+      <c r="AI16">
+        <v>-1</v>
+      </c>
+      <c r="AJ16">
+        <v>1</v>
+      </c>
+      <c r="AK16">
+        <v>-1</v>
+      </c>
+      <c r="AL16">
+        <v>1</v>
       </c>
       <c r="AM16">
         <v>4</v>
@@ -2306,7 +2552,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C17">
         <v>5.5</v>
@@ -2318,7 +2564,7 @@
         <v>-137</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G17">
         <v>824072</v>
@@ -2377,17 +2623,23 @@
       <c r="Y17">
         <v>1.0031</v>
       </c>
+      <c r="Z17">
+        <v>2</v>
+      </c>
       <c r="AA17" t="s">
         <v>44</v>
       </c>
+      <c r="AB17">
+        <v>-0.82</v>
+      </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="AD17">
         <v>4.68</v>
       </c>
       <c r="AE17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF17">
         <v>0.2116</v>
@@ -2397,6 +2649,18 @@
       </c>
       <c r="AH17">
         <v>0</v>
+      </c>
+      <c r="AI17">
+        <v>-2.68</v>
+      </c>
+      <c r="AJ17">
+        <v>2.68</v>
+      </c>
+      <c r="AK17">
+        <v>-2.68</v>
+      </c>
+      <c r="AL17">
+        <v>2.68</v>
       </c>
       <c r="AM17">
         <v>4.68</v>
@@ -2407,10 +2671,10 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G18">
         <v>824152</v>
@@ -2470,16 +2734,16 @@
         <v>0.8828</v>
       </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD18">
         <v>4.17</v>
       </c>
       <c r="AE18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF18">
         <v>0.2198</v>
@@ -2499,7 +2763,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C19">
         <v>4.5</v>
@@ -2511,7 +2775,7 @@
         <v>102</v>
       </c>
       <c r="F19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G19">
         <v>824152</v>
@@ -2570,17 +2834,23 @@
       <c r="Y19">
         <v>1.0194</v>
       </c>
+      <c r="Z19">
+        <v>4</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>-0.5</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD19">
         <v>4</v>
       </c>
       <c r="AE19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF19">
         <v>0.1895</v>
@@ -2589,6 +2859,18 @@
         <v>0.872</v>
       </c>
       <c r="AH19">
+        <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>0</v>
+      </c>
+      <c r="AJ19">
+        <v>0</v>
+      </c>
+      <c r="AK19">
+        <v>0</v>
+      </c>
+      <c r="AL19">
         <v>0</v>
       </c>
       <c r="AM19">
@@ -2600,7 +2882,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C20">
         <v>6.5</v>
@@ -2612,7 +2894,7 @@
         <v>-116</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G20">
         <v>822857</v>
@@ -2671,17 +2953,23 @@
       <c r="Y20">
         <v>1.0791</v>
       </c>
+      <c r="Z20">
+        <v>5</v>
+      </c>
       <c r="AA20" t="s">
         <v>44</v>
       </c>
+      <c r="AB20">
+        <v>1.98</v>
+      </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD20">
         <v>8.48</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.3104</v>
@@ -2691,6 +2979,18 @@
       </c>
       <c r="AH20">
         <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>-3.48</v>
+      </c>
+      <c r="AJ20">
+        <v>3.48</v>
+      </c>
+      <c r="AK20">
+        <v>-3.48</v>
+      </c>
+      <c r="AL20">
+        <v>3.48</v>
       </c>
       <c r="AM20">
         <v>8.48</v>
@@ -2701,7 +3001,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C21">
         <v>6.5</v>
@@ -2713,7 +3013,7 @@
         <v>118</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G21">
         <v>822857</v>
@@ -2772,17 +3072,23 @@
       <c r="Y21">
         <v>1.1182</v>
       </c>
+      <c r="Z21">
+        <v>7</v>
+      </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="AB21">
+        <v>2.6</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="AD21">
         <v>9.1</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
         <v>0.2596</v>
@@ -2792,6 +3098,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>-2.1</v>
+      </c>
+      <c r="AJ21">
+        <v>2.1</v>
+      </c>
+      <c r="AK21">
+        <v>-2.1</v>
+      </c>
+      <c r="AL21">
+        <v>2.1</v>
       </c>
       <c r="AM21">
         <v>9.1</v>
@@ -2802,7 +3120,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C22">
         <v>5.5</v>
@@ -2814,7 +3132,7 @@
         <v>-105</v>
       </c>
       <c r="F22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G22">
         <v>824317</v>
@@ -2873,17 +3191,23 @@
       <c r="Y22">
         <v>1.0239</v>
       </c>
+      <c r="Z22">
+        <v>5</v>
+      </c>
       <c r="AA22" t="s">
         <v>44</v>
       </c>
+      <c r="AB22">
+        <v>1.69</v>
+      </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD22">
         <v>7.19</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.2728</v>
@@ -2893,6 +3217,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>-2.19</v>
+      </c>
+      <c r="AJ22">
+        <v>2.19</v>
+      </c>
+      <c r="AK22">
+        <v>-2.19</v>
+      </c>
+      <c r="AL22">
+        <v>2.19</v>
       </c>
       <c r="AM22">
         <v>7.19</v>
@@ -2903,7 +3239,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C23">
         <v>3.5</v>
@@ -2915,7 +3251,7 @@
         <v>-162</v>
       </c>
       <c r="F23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G23">
         <v>824317</v>
@@ -2974,17 +3310,23 @@
       <c r="Y23">
         <v>0.88</v>
       </c>
+      <c r="Z23">
+        <v>2</v>
+      </c>
       <c r="AA23" t="s">
         <v>44</v>
       </c>
+      <c r="AB23">
+        <v>-1.02</v>
+      </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="AD23">
         <v>2.48</v>
       </c>
       <c r="AE23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF23">
         <v>0.1842</v>
@@ -2994,6 +3336,18 @@
       </c>
       <c r="AH23">
         <v>0</v>
+      </c>
+      <c r="AI23">
+        <v>-0.48</v>
+      </c>
+      <c r="AJ23">
+        <v>0.48</v>
+      </c>
+      <c r="AK23">
+        <v>-0.48</v>
+      </c>
+      <c r="AL23">
+        <v>0.48</v>
       </c>
       <c r="AM23">
         <v>2.48</v>
@@ -3004,7 +3358,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C24">
         <v>3.5</v>
@@ -3016,7 +3370,7 @@
         <v>105</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G24">
         <v>825045</v>
@@ -3075,17 +3429,23 @@
       <c r="Y24">
         <v>0.88</v>
       </c>
+      <c r="Z24">
+        <v>2</v>
+      </c>
       <c r="AA24" t="s">
         <v>44</v>
       </c>
+      <c r="AB24">
+        <v>-0.07</v>
+      </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD24">
         <v>3.43</v>
       </c>
       <c r="AE24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF24">
         <v>0.1806</v>
@@ -3095,6 +3455,18 @@
       </c>
       <c r="AH24">
         <v>0</v>
+      </c>
+      <c r="AI24">
+        <v>-1.43</v>
+      </c>
+      <c r="AJ24">
+        <v>1.43</v>
+      </c>
+      <c r="AK24">
+        <v>-1.43</v>
+      </c>
+      <c r="AL24">
+        <v>1.43</v>
       </c>
       <c r="AM24">
         <v>3.43</v>
@@ -3105,7 +3477,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C25">
         <v>5.5</v>
@@ -3117,7 +3489,7 @@
         <v>-146</v>
       </c>
       <c r="F25" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G25">
         <v>825045</v>
@@ -3176,17 +3548,23 @@
       <c r="Y25">
         <v>1.113</v>
       </c>
+      <c r="Z25">
+        <v>4</v>
+      </c>
       <c r="AA25" t="s">
         <v>44</v>
       </c>
+      <c r="AB25">
+        <v>1.19</v>
+      </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD25">
         <v>6.29</v>
       </c>
       <c r="AE25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AF25">
         <v>0.1749</v>
@@ -3196,6 +3574,18 @@
       </c>
       <c r="AH25">
         <v>0.4</v>
+      </c>
+      <c r="AI25">
+        <v>-2.29</v>
+      </c>
+      <c r="AJ25">
+        <v>2.29</v>
+      </c>
+      <c r="AK25">
+        <v>-2.69</v>
+      </c>
+      <c r="AL25">
+        <v>2.69</v>
       </c>
       <c r="AM25">
         <v>6.69</v>
@@ -3206,7 +3596,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C26">
         <v>5.5</v>
@@ -3218,7 +3608,7 @@
         <v>-148</v>
       </c>
       <c r="F26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G26">
         <v>823262</v>
@@ -3277,17 +3667,23 @@
       <c r="Y26">
         <v>1.0141</v>
       </c>
+      <c r="Z26">
+        <v>7</v>
+      </c>
       <c r="AA26" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="AB26">
+        <v>-0.46</v>
       </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD26">
         <v>5.04</v>
       </c>
       <c r="AE26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF26">
         <v>0.2531</v>
@@ -3297,6 +3693,18 @@
       </c>
       <c r="AH26">
         <v>0</v>
+      </c>
+      <c r="AI26">
+        <v>1.96</v>
+      </c>
+      <c r="AJ26">
+        <v>1.96</v>
+      </c>
+      <c r="AK26">
+        <v>1.96</v>
+      </c>
+      <c r="AL26">
+        <v>1.96</v>
       </c>
       <c r="AM26">
         <v>5.04</v>
@@ -3307,10 +3715,10 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F27" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G27">
         <v>823262</v>
@@ -3370,16 +3778,16 @@
         <v>0.9599</v>
       </c>
       <c r="AA27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD27">
         <v>2.34</v>
       </c>
       <c r="AE27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF27">
         <v>0.1273</v>
@@ -3399,7 +3807,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C28">
         <v>4.5</v>
@@ -3411,7 +3819,7 @@
         <v>-147</v>
       </c>
       <c r="F28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G28">
         <v>823911</v>
@@ -3470,17 +3878,23 @@
       <c r="Y28">
         <v>0.9717</v>
       </c>
+      <c r="Z28">
+        <v>6</v>
+      </c>
       <c r="AA28" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="AB28">
+        <v>-0.68</v>
       </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD28">
         <v>3.82</v>
       </c>
       <c r="AE28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF28">
         <v>0.2082</v>
@@ -3490,6 +3904,18 @@
       </c>
       <c r="AH28">
         <v>0</v>
+      </c>
+      <c r="AI28">
+        <v>2.18</v>
+      </c>
+      <c r="AJ28">
+        <v>2.18</v>
+      </c>
+      <c r="AK28">
+        <v>2.18</v>
+      </c>
+      <c r="AL28">
+        <v>2.18</v>
       </c>
       <c r="AM28">
         <v>3.82</v>
@@ -3500,7 +3926,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C29">
         <v>7.5</v>
@@ -3512,7 +3938,7 @@
         <v>-155</v>
       </c>
       <c r="F29" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G29">
         <v>823911</v>
@@ -3571,17 +3997,23 @@
       <c r="Y29">
         <v>1.0736</v>
       </c>
+      <c r="Z29">
+        <v>9</v>
+      </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="AB29">
+        <v>-0.28</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD29">
         <v>6.82</v>
       </c>
       <c r="AE29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AF29">
         <v>0.2384</v>
@@ -3591,6 +4023,18 @@
       </c>
       <c r="AH29">
         <v>0.4</v>
+      </c>
+      <c r="AI29">
+        <v>2.18</v>
+      </c>
+      <c r="AJ29">
+        <v>2.18</v>
+      </c>
+      <c r="AK29">
+        <v>1.78</v>
+      </c>
+      <c r="AL29">
+        <v>1.78</v>
       </c>
       <c r="AM29">
         <v>7.22</v>
@@ -3601,7 +4045,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C30">
         <v>4.5</v>
@@ -3613,7 +4057,7 @@
         <v>110</v>
       </c>
       <c r="F30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G30">
         <v>823101</v>
@@ -3672,17 +4116,23 @@
       <c r="Y30">
         <v>0.958</v>
       </c>
+      <c r="Z30">
+        <v>3</v>
+      </c>
       <c r="AA30" t="s">
         <v>44</v>
       </c>
+      <c r="AB30">
+        <v>-0.78</v>
+      </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="AD30">
         <v>3.72</v>
       </c>
       <c r="AE30" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF30">
         <v>0.1644</v>
@@ -3692,6 +4142,18 @@
       </c>
       <c r="AH30">
         <v>0</v>
+      </c>
+      <c r="AI30">
+        <v>-0.72</v>
+      </c>
+      <c r="AJ30">
+        <v>0.72</v>
+      </c>
+      <c r="AK30">
+        <v>-0.72</v>
+      </c>
+      <c r="AL30">
+        <v>0.72</v>
       </c>
       <c r="AM30">
         <v>3.72</v>
@@ -3702,7 +4164,7 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C31">
         <v>4.5</v>
@@ -3714,7 +4176,7 @@
         <v>126</v>
       </c>
       <c r="F31" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G31">
         <v>823101</v>
@@ -3773,17 +4235,23 @@
       <c r="Y31">
         <v>0.889</v>
       </c>
+      <c r="Z31">
+        <v>6</v>
+      </c>
       <c r="AA31" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="AB31">
+        <v>-0.1</v>
       </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD31">
         <v>4.4</v>
       </c>
       <c r="AE31" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AF31">
         <v>0.2182</v>
@@ -3793,6 +4261,18 @@
       </c>
       <c r="AH31">
         <v>0</v>
+      </c>
+      <c r="AI31">
+        <v>1.6</v>
+      </c>
+      <c r="AJ31">
+        <v>1.6</v>
+      </c>
+      <c r="AK31">
+        <v>1.6</v>
+      </c>
+      <c r="AL31">
+        <v>1.6</v>
       </c>
       <c r="AM31">
         <v>4.4</v>
@@ -3803,7 +4283,7 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32">
         <v>7.5</v>
@@ -3815,31 +4295,31 @@
         <v>-130</v>
       </c>
       <c r="F32" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L32">
         <v>6</v>
       </c>
       <c r="S32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:39" x14ac:dyDescent="0.25">
@@ -3847,7 +4327,7 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C33">
         <v>4.5</v>
@@ -3859,31 +4339,31 @@
         <v>-102</v>
       </c>
       <c r="F33" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L33">
         <v>5</v>
       </c>
       <c r="S33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:39" x14ac:dyDescent="0.25">
@@ -3891,7 +4371,7 @@
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C34">
         <v>2.5</v>
@@ -3903,31 +4383,31 @@
         <v>127</v>
       </c>
       <c r="F34" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L34">
         <v>3</v>
       </c>
       <c r="S34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>